<commit_message>
class 13 excel reader
</commit_message>
<xml_diff>
--- a/Files/Employees.xlsx
+++ b/Files/Employees.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>First Name</t>
   </si>
@@ -43,6 +43,15 @@
   </si>
   <si>
     <t>Salary</t>
+  </si>
+  <si>
+    <t>Muhammad</t>
+  </si>
+  <si>
+    <t>Ali</t>
+  </si>
+  <si>
+    <t>Madina</t>
   </si>
   <si>
     <t>John</t>
@@ -1247,8 +1256,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelRow="5" outlineLevelCol="4"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="13.7890625" customWidth="1"/>
   </cols>
@@ -1278,13 +1287,13 @@
         <v>6</v>
       </c>
       <c r="C2">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
       </c>
       <c r="E2">
-        <v>55000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1295,13 +1304,13 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
       </c>
       <c r="E3">
-        <v>67000</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1312,13 +1321,13 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
       </c>
       <c r="E4">
-        <v>72000</v>
+        <v>67000</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1329,13 +1338,13 @@
         <v>15</v>
       </c>
       <c r="C5">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
       </c>
       <c r="E5">
-        <v>48000</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1346,12 +1355,29 @@
         <v>18</v>
       </c>
       <c r="C6">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
         <v>19</v>
       </c>
       <c r="E6">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7">
         <v>61000</v>
       </c>
     </row>

</xml_diff>